<commit_message>
se agregan los ultimos cambios para el modelo 3 ;a parte de transacciones se anade xpath dinamico y otros ajustes menores
</commit_message>
<xml_diff>
--- a/Banca en Linea modelo 3/Datos/Datos.xlsx
+++ b/Banca en Linea modelo 3/Datos/Datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bespinosa\Documents\Katalon\Demo Banca en Linea\Demo-Banca-en-Linea\Banca en Linea modelo 3\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E136D278-3276-4933-9EEA-94D7C94E4AC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B87B3397-CC43-4978-A9EB-34ACE160EDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>prueba</t>
   </si>
@@ -64,6 +64,15 @@
   </si>
   <si>
     <t>Qaz12345</t>
+  </si>
+  <si>
+    <t>tipo_producto</t>
+  </si>
+  <si>
+    <t>CUENTA DE AHORRO</t>
+  </si>
+  <si>
+    <t>cuenta_destino</t>
   </si>
 </sst>
 </file>
@@ -393,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
@@ -402,9 +411,11 @@
     <col min="5" max="5" width="22.08984375" customWidth="1"/>
     <col min="6" max="6" width="24.81640625" customWidth="1"/>
     <col min="7" max="7" width="46.6328125" customWidth="1"/>
+    <col min="8" max="8" width="19.08984375" customWidth="1"/>
+    <col min="9" max="9" width="19.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -426,8 +437,14 @@
       <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -448,6 +465,12 @@
       </c>
       <c r="G2" s="4" t="s">
         <v>9</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="3">
+        <v>4010324099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>